<commit_message>
Add new docs User stories and Flow chart
</commit_message>
<xml_diff>
--- a/Documents/JO User Story Excel Version_04202026.xlsx
+++ b/Documents/JO User Story Excel Version_04202026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unitedlaboratoriesinc-my.sharepoint.com/personal/mbferrer_unilab_com_ph/Documents/5 TA PROJECTS/Job Offer Tool/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitLab\joboffer\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="88" documentId="8_{E62D68F4-B4D8-43CD-9094-2E18998D019F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA024A70-34D9-45E2-B88E-80B94EAB085F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFE57591-61E9-46ED-8D1A-58E081B279E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_Epic_Overview" sheetId="1" r:id="rId1"/>
@@ -1374,10 +1374,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>